<commit_message>
Dados IMEA de 28/07/2026
</commit_message>
<xml_diff>
--- a/dados/imea_boi.xlsx
+++ b/dados/imea_boi.xlsx
@@ -1,33 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Indice" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOI GORDO A VISTA" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VACA GORDA A VISTA" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ESCALA DE ABATE" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOI GORDO A PRAZO" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VACA GORDA A PRAZO" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOI MAGRO NELORE 360KG 12@" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GARROTE NELORE 18M 285 KG 9,5@" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BEZERRO NELORE DE 12M 210KG 7@" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BEZERRO NELORE 8M 165KG 5,5@" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VACA NELORE 315 KG 10,5@" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOVILHA NELORE 18M 255KG 8,5@" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BEZERRA NELORE 12M 180KG 6@" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BEZERRA NELORE 8M 150KG 5@" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOURINHO NELORE 22@" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VACA NELORE PARIDA 12,5@" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CORTES NO ATACADO" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ABATE MACHOS" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ABATE FEMEAS" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UTL CAP FRIGORIFICA - TOTAL" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REBANHO TOTAL" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="_Indice" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="BOI GORDO A VISTA" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="VACA GORDA A VISTA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ESCALA DE ABATE" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="BOI GORDO A PRAZO" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="VACA GORDA A PRAZO" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="BOI MAGRO NELORE 360KG 12@" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="GARROTE NELORE 18M 285 KG 9,5@" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="BEZERRO NELORE DE 12M 210KG 7@" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="BEZERRO NELORE 8M 165KG 5,5@" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="VACA NELORE 315 KG 10,5@" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="NOVILHA NELORE 18M 255KG 8,5@" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="BEZERRA NELORE 12M 180KG 6@" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="BEZERRA NELORE 8M 150KG 5@" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="TOURINHO NELORE 22@" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="VACA NELORE PARIDA 12,5@" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="CORTES NO ATACADO" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="ABATE MACHOS" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="ABATE FEMEAS" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="UTL CAP FRIGORIFICA - TOTAL" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="REBANHO TOTAL" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>